<commit_message>
#137 Client and JLCPCB BOM updated
</commit_message>
<xml_diff>
--- a/Design-Files/ArmBand-Sensor-Board-v2.0/BOM/Client_BOM_ArmBand-Sensor-Board.xlsx
+++ b/Design-Files/ArmBand-Sensor-Board-v2.0/BOM/Client_BOM_ArmBand-Sensor-Board.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ManarHarake-sEMGDevice\Design-Files\ArmBand-Sensor-Board-v1.0\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ManarHarake-sEMGDevice\Design-Files\ArmBand-Sensor-Board-v2.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="68">
   <si>
     <t>#</t>
   </si>
@@ -213,26 +213,23 @@
     <t>Quantity</t>
   </si>
   <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
     <t>Value</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>Remarks</t>
-  </si>
-  <si>
-    <t>Custom</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solder Bridge </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -275,6 +272,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -391,7 +395,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -430,6 +434,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -770,13 +780,13 @@
         <v>49</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>63</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -868,7 +878,7 @@
         <v>52</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
@@ -946,30 +956,30 @@
         <v>6</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="D8" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="F8" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="G8" s="9" t="s">
+      <c r="F8" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="G8" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="H8" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="I8" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="J8" s="9">
+      <c r="H8" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="I8" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="J8" s="15">
         <v>6</v>
       </c>
-      <c r="K8" s="9"/>
+      <c r="K8" s="15"/>
     </row>
     <row r="9" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -995,8 +1005,8 @@
       <c r="H9" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="I9" s="10" t="s">
-        <v>65</v>
+      <c r="I9" s="8" t="s">
+        <v>64</v>
       </c>
       <c r="J9" s="7">
         <v>2</v>
@@ -1028,7 +1038,7 @@
         <v>56</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -1059,8 +1069,8 @@
       <c r="H11" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="I11" s="10" t="s">
-        <v>65</v>
+      <c r="I11" s="8" t="s">
+        <v>64</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
@@ -1092,7 +1102,7 @@
         <v>58</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J12" s="9">
         <v>2</v>

</xml_diff>